<commit_message>
Finalize Level 1 lessons 1.1, 1.2, 1.3, 1.5, 1.6 (reviewed and verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/01-foundations/03-formatting-cells/1.3-formatting-cells.xlsx
+++ b/01-foundations/03-formatting-cells/1.3-formatting-cells.xlsx
@@ -1100,7 +1100,7 @@
     <row r="1">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>Bluestone Memorial Hospital · 2025 Operating Expense Budget vs Actual by Department</t>
+          <t>Bluestone Memorial Hospital · 2025 Expense Budget vs Actual</t>
         </is>
       </c>
       <c r="B1" s="43" t="n"/>
@@ -2246,7 +2246,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="66" customHeight="1">
+    <row r="16" ht="81" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>11</t>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Column G (LOS vs Expected) stores LOS minus the diagnosis's expected LOS, in days. Write a two-section custom format for G5:G40: positive values in red with a plus sign and the word days (like +2.1 days), and negative values with a minus sign (like -0.4 days), each with one decimal. What does G5 display?</t>
+          <t>Column G (LOS vs Expected) stores LOS minus the diagnosis's expected LOS, in days, so a positive value means the patient stayed longer than expected. Write a two-section custom format for G5:G40: positive values in red with a plus sign and the word days (like +2.1 days), and negative values with a minus sign (like -0.4 days), each with one decimal. What does G5 display?</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Finish the Budget report so it looks like the hidden Budget Key sheet: (1) unmerge A1:F1 and center the title with Center Across Selection; (2) unmerge column A and fill each service line down so every row has its label; (3) make header row 4 bold with white text on a dark blue fill, wrapped and centered; (4) add All Borders to A4:F21; (5) apply the Total cell style to A21:F21; (6) select A4:F21 and AutoFit the columns with Home → Format → AutoFit Column Width. Then zoom in on row 21: what kind of line does the Total style draw along the bottom of the row?</t>
+          <t>Finish the Budget report so it looks like the hidden Budget Key sheet: (1) unmerge A1:F1 and center the title with Center Across Selection; (2) unmerge column A and fill each service line down so every row has its label; (3) make header row 4 bold with white text on a dark blue fill, wrapped and centered; (4) add All Borders to A4:F21; (5) apply the Total cell style to A21:F21; (6) select A4:F21 and AutoFit the columns with Home → Format → AutoFit Column Width. Then zoom in on row 21: what kind of line does the Total style draw along the bottom of the row? Answer in a word or two.</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D18" s="21" t="n"/>
       <c r="E18" s="22">
-        <f>IF(IFERROR(D18="",FALSE),"",IF(IFERROR(OR(LOWER(TRIM(D18&amp;""))=LOWER(TRIM('Answer Key'!$C$17&amp;"")),LOWER(TRIM(D18&amp;""))="double line",LOWER(TRIM(D18&amp;""))="a double line",LOWER(TRIM(D18&amp;""))="double border",LOWER(TRIM(D18&amp;""))="a double border",LOWER(TRIM(D18&amp;""))="double bottom border",LOWER(TRIM(D18&amp;""))="double underline",LOWER(TRIM(D18&amp;""))="double-line",LOWER(TRIM(D18&amp;""))="two lines",LOWER(TRIM(D18&amp;""))="2 lines",LOWER(TRIM(D18&amp;""))="double lines"),FALSE),"✔ Correct","✘ Not yet"))</f>
+        <f>IF(IFERROR(D18="",FALSE),"",IF(IFERROR(OR(LOWER(TRIM(D18&amp;""))=LOWER(TRIM('Answer Key'!$C$17&amp;"")),LOWER(TRIM(D18&amp;""))="double line",LOWER(TRIM(D18&amp;""))="a double line",LOWER(TRIM(D18&amp;""))="double border",LOWER(TRIM(D18&amp;""))="a double border",LOWER(TRIM(D18&amp;""))="double bottom border",LOWER(TRIM(D18&amp;""))="a double bottom border",LOWER(TRIM(D18&amp;""))="bottom double border",LOWER(TRIM(D18&amp;""))="double line border",LOWER(TRIM(D18&amp;""))="double underline",LOWER(TRIM(D18&amp;""))="double-line",LOWER(TRIM(D18&amp;""))="two lines",LOWER(TRIM(D18&amp;""))="2 lines",LOWER(TRIM(D18&amp;""))="double lines"),FALSE),"✔ Correct","✘ Not yet"))</f>
         <v/>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
     <row r="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>Bluestone Memorial Hospital · 2025 Operating Expense Budget vs Actual by Department</t>
+          <t>Bluestone Memorial Hospital · 2025 Expense Budget vs Actual</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
     <row r="2" ht="184" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>The Emergency Department director presents the December 2025 operating report to the CFO next week. Finance's style guide has five rules for department reports. Apply them on the Dec Report sheet, writing every custom format code yourself, then type what each listed cell displays. When you finish, compare your sheet with the hidden Report Key sheet.
+          <t>The Emergency Department director presents the December 2025 operating report to the CFO next week. Finance's style guide has five rules for department reports. Apply them on the Dec Report sheet, writing every custom format code yourself. Then type what each listed Dec Report cell displays into the yellow cells on the Bonus sheet. When you finish, compare your sheet with the hidden Report Key sheet.
 - Rule 1: Center the title across A1:I1 without merging. Make the header row bold white text on a dark blue fill, wrapped and centered. Give the Total row the Total cell style.
 - Rule 2: Show Dec Budget and Dec Actual in thousands with one decimal place, a dollar sign, and a K, so 843,879 displays as $843.9K.
 - Rule 3: Show both Variance columns the same way, except that negative variances (over budget) are red and in parentheses instead of having a minus sign, so -25,403 displays as ($25.4K).
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Rule 2: what does C5 (Employee Benefits, Dec Actual) display?</t>
+          <t>Rule 2: on the Dec Report sheet, what does C5 (Employee Benefits, Dec Actual) display?</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Rule 3: what does D11 (Salaries &amp; Wages, Dec Variance) display?</t>
+          <t>Rule 3: on the Dec Report sheet, what does D11 (Salaries &amp; Wages, Dec Variance) display?</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Rule 4: what does I6 (Equipment &amp; Maintenance, YTD Var %) display?</t>
+          <t>Rule 4: on the Dec Report sheet, what does I6 (Equipment &amp; Maintenance, YTD Var %) display?</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Rule 5: what does G12 (the Total row's YTD Actual) display?</t>
+          <t>Rule 5: on the Dec Report sheet, what does G12 (the Total row's YTD Actual) display?</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Rule 5: what does F8 (Other Operating, YTD Budget) display?</t>
+          <t>Rule 5: on the Dec Report sheet, what does F8 (Other Operating, YTD Budget) display?</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -4934,7 +4934,7 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Column G (LOS vs Expected) stores LOS minus the diagnosis's expected LOS, in days. Write a two-section custom format for G5:G40: positive values in red with a plus sign and the word days (like +2.1 days), and negative values with a minus sign (like -0.4 days), each with one decimal. What does G5 display?</t>
+          <t>Column G (LOS vs Expected) stores LOS minus the diagnosis's expected LOS, in days, so a positive value means the patient stayed longer than expected. Write a two-section custom format for G5:G40: positive values in red with a plus sign and the word days (like +2.1 days), and negative values with a minus sign (like -0.4 days), each with one decimal. What does G5 display?</t>
         </is>
       </c>
       <c r="C15" s="37" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Finish the Budget report so it looks like the hidden Budget Key sheet: (1) unmerge A1:F1 and center the title with Center Across Selection; (2) unmerge column A and fill each service line down so every row has its label; (3) make header row 4 bold with white text on a dark blue fill, wrapped and centered; (4) add All Borders to A4:F21; (5) apply the Total cell style to A21:F21; (6) select A4:F21 and AutoFit the columns with Home → Format → AutoFit Column Width. Then zoom in on row 21: what kind of line does the Total style draw along the bottom of the row?</t>
+          <t>Finish the Budget report so it looks like the hidden Budget Key sheet: (1) unmerge A1:F1 and center the title with Center Across Selection; (2) unmerge column A and fill each service line down so every row has its label; (3) make header row 4 bold with white text on a dark blue fill, wrapped and centered; (4) add All Borders to A4:F21; (5) apply the Total cell style to A21:F21; (6) select A4:F21 and AutoFit the columns with Home → Format → AutoFit Column Width. Then zoom in on row 21: what kind of line does the Total style draw along the bottom of the row? Answer in a word or two.</t>
         </is>
       </c>
       <c r="C17" s="37" t="inlineStr">
@@ -5484,7 +5484,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="51" customHeight="1">
+    <row r="5" ht="171" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Rule 2: what does C5 (Employee Benefits, Dec Actual) display?</t>
+          <t>Rule 2: on the Dec Report sheet, what does C5 (Employee Benefits, Dec Actual) display?</t>
         </is>
       </c>
       <c r="C5" s="37" t="inlineStr">
@@ -5502,7 +5502,9 @@
       </c>
       <c r="D5" s="38" t="inlineStr">
         <is>
-          <t>Select **'Dec Report'!B5:C12**, press **Ctrl + 1** (Mac: **⌘ + 1**), choose **Custom**, and type `$#,##0.0,"K"`.</t>
+          <t>1. **Rule 1** uses the same steps as practice task 13: select **'Dec Report'!A1:I1** and set **Center Across Selection** (**Ctrl + 1**, Mac: **⌘ + 1** → **Alignment** tab), style the header **A4:I4** (bold, white font, dark blue fill, Wrap Text, Center), and apply **Home → Cell Styles → Total** to **A12:I12**.
+2. **Rule 2:** select **'Dec Report'!B5:C12**, press **Ctrl + 1** (Mac: **⌘ + 1**), choose **Custom**, and type `$#,##0.0,"K"`.
+3. Read **C5**.</t>
         </is>
       </c>
       <c r="E5" cm="1" s="39">
@@ -5523,7 +5525,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Rule 3: what does D11 (Salaries &amp; Wages, Dec Variance) display?</t>
+          <t>Rule 3: on the Dec Report sheet, what does D11 (Salaries &amp; Wages, Dec Variance) display?</t>
         </is>
       </c>
       <c r="C6" s="37" t="inlineStr">
@@ -5533,7 +5535,7 @@
       </c>
       <c r="D6" s="38" t="inlineStr">
         <is>
-          <t>Select **'Dec Report'!D5:D12**, then Ctrl+click **H5:H12**. Apply the custom format `$#,##0.0,"K";[Red]($#,##0.0,"K")`.</t>
+          <t>Select **'Dec Report'!D5:D12**, then hold **Ctrl** (Mac: **⌘**) and drag over **H5:H12** to add the YTD Variance column. Apply the custom format `$#,##0.0,"K";[Red]($#,##0.0,"K")`.</t>
         </is>
       </c>
       <c r="E6" cm="1" s="39">
@@ -5554,7 +5556,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Rule 4: what does I6 (Equipment &amp; Maintenance, YTD Var %) display?</t>
+          <t>Rule 4: on the Dec Report sheet, what does I6 (Equipment &amp; Maintenance, YTD Var %) display?</t>
         </is>
       </c>
       <c r="C7" s="37" t="inlineStr">
@@ -5564,7 +5566,7 @@
       </c>
       <c r="D7" s="38" t="inlineStr">
         <is>
-          <t>Select **'Dec Report'!E5:E12** and Ctrl+click **I5:I12**. Apply the custom format `0.0%;[Red](0.0%)`.</t>
+          <t>Select **'Dec Report'!E5:E12**, then hold **Ctrl** (Mac: **⌘**) and drag over **I5:I12**. Apply the custom format `0.0%;[Red](0.0%)`.</t>
         </is>
       </c>
       <c r="E7" cm="1" s="39">
@@ -5585,7 +5587,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Rule 5: what does G12 (the Total row's YTD Actual) display?</t>
+          <t>Rule 5: on the Dec Report sheet, what does G12 (the Total row's YTD Actual) display?</t>
         </is>
       </c>
       <c r="C8" s="37" t="inlineStr">
@@ -5616,7 +5618,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Rule 5: what does F8 (Other Operating, YTD Budget) display?</t>
+          <t>Rule 5: on the Dec Report sheet, what does F8 (Other Operating, YTD Budget) display?</t>
         </is>
       </c>
       <c r="C9" s="37" t="inlineStr">

</xml_diff>